<commit_message>
cdi-board: TopB 2 (silkscreen REV 1.0) - BOM
Imported from original project folder:
  FPGA_TopVtester2

29 files changed, 613294 insertions(+), 23130 deletions(-)
</commit_message>
<xml_diff>
--- a/hardware/cdi-board/BOM.xlsx
+++ b/hardware/cdi-board/BOM.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="374">
   <si>
     <t>478-1746-1-ND</t>
   </si>
@@ -855,9 +855,6 @@
     <t>Have instock from Ebay LM1117 3.3</t>
   </si>
   <si>
-    <t>887-1013-ND</t>
-  </si>
-  <si>
     <t>12MHz ±30ppm Crystal 18pF HC49/US</t>
   </si>
   <si>
@@ -867,9 +864,6 @@
     <t>IC FLASH 2MBIT 75MHZ 8SO</t>
   </si>
   <si>
-    <t>M25P80-VMN6TPCT-ND</t>
-  </si>
-  <si>
     <t>IC FLASH 8MBIT 75MHZ 8SO</t>
   </si>
   <si>
@@ -961,13 +955,196 @@
   </si>
   <si>
     <t>X1</t>
+  </si>
+  <si>
+    <t>631-1105-ND</t>
+  </si>
+  <si>
+    <t>296-12896-5-ND</t>
+  </si>
+  <si>
+    <t>74HC27</t>
+  </si>
+  <si>
+    <t>U72</t>
+  </si>
+  <si>
+    <t>296-12892-5-ND</t>
+  </si>
+  <si>
+    <t>U19</t>
+  </si>
+  <si>
+    <t>74HC20</t>
+  </si>
+  <si>
+    <t>74HC32</t>
+  </si>
+  <si>
+    <t>296-1589-5-ND</t>
+  </si>
+  <si>
+    <t>U5 U71 U81</t>
+  </si>
+  <si>
+    <t>296-2138-5-ND</t>
+  </si>
+  <si>
+    <t>74HCT93</t>
+  </si>
+  <si>
+    <t>U15</t>
+  </si>
+  <si>
+    <t>296-1568-5-ND</t>
+  </si>
+  <si>
+    <t>U79</t>
+  </si>
+  <si>
+    <t>74HC05</t>
+  </si>
+  <si>
+    <t>296-9196-5-ND</t>
+  </si>
+  <si>
+    <t>74HC30</t>
+  </si>
+  <si>
+    <t>U90</t>
+  </si>
+  <si>
+    <t>296-9240-5-ND</t>
+  </si>
+  <si>
+    <t>74HC75</t>
+  </si>
+  <si>
+    <t>296-8257-5-ND</t>
+  </si>
+  <si>
+    <t>U18</t>
+  </si>
+  <si>
+    <t>74HC175</t>
+  </si>
+  <si>
+    <t>296-1591-5-ND</t>
+  </si>
+  <si>
+    <t>U9 U73 U74 U75</t>
+  </si>
+  <si>
+    <t>74HC373</t>
+  </si>
+  <si>
+    <t>74HC240</t>
+  </si>
+  <si>
+    <t>296-1580-5-ND</t>
+  </si>
+  <si>
+    <t>U56</t>
+  </si>
+  <si>
+    <t>1450-1027-ND</t>
+  </si>
+  <si>
+    <t>AS6C4008-55PCN</t>
+  </si>
+  <si>
+    <t>U10, U11, U12, U13</t>
+  </si>
+  <si>
+    <t>U2, U3, U4, U5, U6</t>
+  </si>
+  <si>
+    <t>U9</t>
+  </si>
+  <si>
+    <t>U26, U41</t>
+  </si>
+  <si>
+    <t>74LS07</t>
+  </si>
+  <si>
+    <t>U14</t>
+  </si>
+  <si>
+    <t>U27</t>
+  </si>
+  <si>
+    <t>U20</t>
+  </si>
+  <si>
+    <t>296-4290-5-ND</t>
+  </si>
+  <si>
+    <t>74AC04</t>
+  </si>
+  <si>
+    <t>296-4301-5-ND</t>
+  </si>
+  <si>
+    <t>74AC14</t>
+  </si>
+  <si>
+    <t>296-4315-5-ND</t>
+  </si>
+  <si>
+    <t>74AC245</t>
+  </si>
+  <si>
+    <t>296-26376-5-ND</t>
+  </si>
+  <si>
+    <t>74AC373</t>
+  </si>
+  <si>
+    <t>296-1566-5-ND</t>
+  </si>
+  <si>
+    <t>74HC04</t>
+  </si>
+  <si>
+    <t>296-8214-5-ND</t>
+  </si>
+  <si>
+    <t>74HC10</t>
+  </si>
+  <si>
+    <t>296-8230-5-ND</t>
+  </si>
+  <si>
+    <t>74HC139</t>
+  </si>
+  <si>
+    <t>296-8248-5-ND</t>
+  </si>
+  <si>
+    <t>74HC164</t>
+  </si>
+  <si>
+    <t>296-8357-5-ND</t>
+  </si>
+  <si>
+    <t>74HC682</t>
+  </si>
+  <si>
+    <t>U17, U40</t>
+  </si>
+  <si>
+    <t>U23, U28, U29, U30, U31</t>
+  </si>
+  <si>
+    <t>1265-1133-1-ND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1006,6 +1183,19 @@
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1080,7 +1270,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1090,6 +1280,19 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="4"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -1388,7 +1591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2042,10 +2245,10 @@
         <v>260</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D45">
         <v>2</v>
@@ -2069,11 +2272,11 @@
       <c r="A47" t="s">
         <v>268</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C47" t="s">
         <v>279</v>
-      </c>
-      <c r="C47" t="s">
-        <v>280</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -2084,10 +2287,10 @@
         <v>252</v>
       </c>
       <c r="B48" t="s">
+        <v>280</v>
+      </c>
+      <c r="C48" t="s">
         <v>281</v>
-      </c>
-      <c r="C48" t="s">
-        <v>282</v>
       </c>
       <c r="D48">
         <v>2</v>
@@ -2097,11 +2300,11 @@
       <c r="A49" t="s">
         <v>252</v>
       </c>
-      <c r="B49" t="s">
-        <v>283</v>
+      <c r="B49" s="7" t="s">
+        <v>373</v>
       </c>
       <c r="C49" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D49">
         <v>2</v>
@@ -2112,10 +2315,10 @@
         <v>242</v>
       </c>
       <c r="B50" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C50" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D50">
         <v>5</v>
@@ -2129,10 +2332,10 @@
         <v>64</v>
       </c>
       <c r="B51" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C51" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D51">
         <v>5</v>
@@ -2143,7 +2346,7 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B52" t="s">
         <v>15</v>
@@ -2163,10 +2366,10 @@
         <v>237</v>
       </c>
       <c r="B53" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C53" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D53">
         <v>10</v>
@@ -2180,10 +2383,10 @@
         <v>235</v>
       </c>
       <c r="B54" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C54" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D54">
         <v>5</v>
@@ -2231,10 +2434,10 @@
         <v>229</v>
       </c>
       <c r="B57" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C57" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D57">
         <v>5</v>
@@ -2248,10 +2451,10 @@
         <v>7</v>
       </c>
       <c r="B58" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C58" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D58">
         <v>2</v>
@@ -2262,7 +2465,7 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B59" t="s">
         <v>176</v>
@@ -2280,24 +2483,349 @@
     <row r="61" spans="1:6" ht="15.75" thickBot="1"/>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
+        <v>312</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="F62" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="16.5" customHeight="1"/>
+    <row r="67" spans="1:4">
+      <c r="A67" t="s">
+        <v>316</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D62">
-        <v>1</v>
-      </c>
-      <c r="F62" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="16.5" customHeight="1"/>
+      <c r="C67" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="D67">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" t="s">
+        <v>318</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="D68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" t="s">
+        <v>322</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="D69">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" t="s">
+        <v>325</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="D70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" t="s">
+        <v>327</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="D71">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" t="s">
+        <v>331</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="D72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" t="s">
+        <v>92</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D73">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" t="s">
+        <v>335</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" t="s">
+        <v>338</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="D75">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" t="s">
+        <v>342</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="D76">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" t="s">
+        <v>325</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="D78">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="C83" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="D83" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C84" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="D84" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="C85" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="D85" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C86" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="D86" s="10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="B87" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="C87" s="11" t="s">
+        <v>362</v>
+      </c>
+      <c r="D87" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="B88" s="11"/>
+      <c r="C88" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="D88" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="C89" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="D89" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C90" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="D90" s="10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" s="8"/>
+      <c r="B91" s="11"/>
+      <c r="C91" s="11"/>
+      <c r="D91" s="10"/>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C92" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="D92" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="C93" s="11" t="s">
+        <v>368</v>
+      </c>
+      <c r="D93" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="C94" s="11" t="s">
+        <v>370</v>
+      </c>
+      <c r="D94" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" s="8"/>
+      <c r="B95" s="9"/>
+      <c r="C95" s="9"/>
+      <c r="D95" s="10"/>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" s="8"/>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9"/>
+      <c r="D96" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3032,13 +3560,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>126</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3049,13 +3577,13 @@
         <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>162</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -3080,7 +3608,7 @@
         <v>201</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -3237,7 +3765,7 @@
         <v>223</v>
       </c>
       <c r="D22" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -3273,7 +3801,7 @@
         <v>228</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -3298,10 +3826,10 @@
         <v>230</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -3315,10 +3843,10 @@
         <v>231</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -3332,7 +3860,7 @@
         <v>232</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>

</xml_diff>